<commit_message>
2023-06-20   Lambda  修改PLM 已知问题
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-plm/src/main/resources/excel/product.xlsx
+++ b/erp-server/erp-server-plm/src/main/resources/excel/product.xlsx
@@ -62,10 +62,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{.isAddProductnName}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>{.grade}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -130,10 +126,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>计划工时(h)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>创建时间</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -207,6 +199,14 @@
   </si>
   <si>
     <t>{.createUserName}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>计划工时</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.isAddProductName}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -642,55 +642,55 @@
         <v>2</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="J1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="W1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:24" s="5" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.15">
@@ -707,64 +707,64 @@
         <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="H2" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="O2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="P2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="O2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="S2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="T2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="R2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="S2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="X2" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.15">

</xml_diff>